<commit_message>
Sep 2025 data update
</commit_message>
<xml_diff>
--- a/data/BEA/bea_const_price_indices.xlsx
+++ b/data/BEA/bea_const_price_indices.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="114">
   <si>
     <t xml:space="preserve">Table 5.3.4. Price Indexes for Private Fixed Investment by Type</t>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Bureau of Economic Analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">Last Revised on: April 30, 2025 - Next Release Date May 29, 2025</t>
+    <t xml:space="preserve">Last Revised on: August 28, 2025 - Next Release Date September 25, 2025</t>
   </si>
   <si>
     <t xml:space="preserve">Line</t>
@@ -555,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:EB49"/>
+  <dimension ref="A1:EC49"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.85" bestFit="1" customWidth="1" collapsed="1"/>
@@ -688,7 +688,8 @@
     <col min="128" max="128" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="129" max="129" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="130" max="130" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="131" max="131" width="7.800000000000001" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="131" max="131" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="132" max="132" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -914,6 +915,7 @@
       <c r="EA6" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="EB6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="1"/>
@@ -1305,6 +1307,9 @@
       <c r="EA7" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="EB7" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
@@ -1698,7 +1703,10 @@
         <v>123.666</v>
       </c>
       <c r="EA8" s="4">
-        <v>124.041</v>
+        <v>124.042</v>
+      </c>
+      <c r="EB8" s="4">
+        <v>123.993</v>
       </c>
     </row>
     <row r="9">
@@ -2093,7 +2101,10 @@
         <v>115.98</v>
       </c>
       <c r="EA9" s="4">
-        <v>116.109</v>
+        <v>116.094</v>
+      </c>
+      <c r="EB9" s="4">
+        <v>115.943</v>
       </c>
     </row>
     <row r="10">
@@ -2488,7 +2499,10 @@
         <v>135.041</v>
       </c>
       <c r="EA10" s="4">
-        <v>135.419</v>
+        <v>135.879</v>
+      </c>
+      <c r="EB10" s="4">
+        <v>135.629</v>
       </c>
     </row>
     <row r="11">
@@ -2883,7 +2897,10 @@
         <v>156.951</v>
       </c>
       <c r="EA11" s="0">
-        <v>158.1</v>
+        <v>158.351</v>
+      </c>
+      <c r="EB11" s="0">
+        <v>157.877</v>
       </c>
     </row>
     <row r="12">
@@ -3278,7 +3295,10 @@
         <v>156.648</v>
       </c>
       <c r="EA12" s="0">
-        <v>157.933</v>
+        <v>157.793</v>
+      </c>
+      <c r="EB12" s="0">
+        <v>158.166</v>
       </c>
     </row>
     <row r="13">
@@ -3673,7 +3693,10 @@
         <v>121.064</v>
       </c>
       <c r="EA13" s="0">
-        <v>120.701</v>
+        <v>120.692</v>
+      </c>
+      <c r="EB13" s="0">
+        <v>121.194</v>
       </c>
     </row>
     <row r="14">
@@ -4068,7 +4091,10 @@
         <v>90.835</v>
       </c>
       <c r="EA14" s="0">
-        <v>89.18</v>
+        <v>91.544</v>
+      </c>
+      <c r="EB14" s="0">
+        <v>89.036</v>
       </c>
     </row>
     <row r="15">
@@ -4463,7 +4489,10 @@
         <v>136.7</v>
       </c>
       <c r="EA15" s="0">
-        <v>137.472</v>
+        <v>137.817</v>
+      </c>
+      <c r="EB15" s="0">
+        <v>138.144</v>
       </c>
     </row>
     <row r="16">
@@ -4858,7 +4887,10 @@
         <v>114.017</v>
       </c>
       <c r="EA16" s="4">
-        <v>114.18</v>
+        <v>114.23</v>
+      </c>
+      <c r="EB16" s="4">
+        <v>115.028</v>
       </c>
     </row>
     <row r="17">
@@ -5253,7 +5285,10 @@
         <v>97.603</v>
       </c>
       <c r="EA17" s="0">
-        <v>97.834</v>
+        <v>97.918</v>
+      </c>
+      <c r="EB17" s="0">
+        <v>98.33</v>
       </c>
     </row>
     <row r="18">
@@ -5650,6 +5685,9 @@
       <c r="EA18" s="0">
         <v>102.902</v>
       </c>
+      <c r="EB18" s="0">
+        <v>102.799</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
@@ -6043,7 +6081,10 @@
         <v>95.619</v>
       </c>
       <c r="EA19" s="0">
-        <v>95.815</v>
+        <v>95.945</v>
+      </c>
+      <c r="EB19" s="0">
+        <v>96.68</v>
       </c>
     </row>
     <row r="20">
@@ -6438,7 +6479,10 @@
         <v>126.089</v>
       </c>
       <c r="EA20" s="0">
-        <v>126.909</v>
+        <v>127.022</v>
+      </c>
+      <c r="EB20" s="0">
+        <v>128.438</v>
       </c>
     </row>
     <row r="21">
@@ -6833,7 +6877,10 @@
         <v>114.777</v>
       </c>
       <c r="EA21" s="0">
-        <v>114.103</v>
+        <v>114.106</v>
+      </c>
+      <c r="EB21" s="0">
+        <v>114.821</v>
       </c>
     </row>
     <row r="22">
@@ -7228,7 +7275,10 @@
         <v>130.255</v>
       </c>
       <c r="EA22" s="0">
-        <v>130.632</v>
+        <v>130.583</v>
+      </c>
+      <c r="EB22" s="0">
+        <v>131.708</v>
       </c>
     </row>
     <row r="23">
@@ -7623,7 +7673,10 @@
         <v>109.033</v>
       </c>
       <c r="EA23" s="4">
-        <v>109.021</v>
+        <v>108.735</v>
+      </c>
+      <c r="EB23" s="4">
+        <v>107.763</v>
       </c>
     </row>
     <row r="24">
@@ -8018,7 +8071,10 @@
         <v>92.241</v>
       </c>
       <c r="EA24" s="0">
-        <v>91.092</v>
+        <v>90.559</v>
+      </c>
+      <c r="EB24" s="0">
+        <v>87.662</v>
       </c>
     </row>
     <row r="25">
@@ -8415,6 +8471,9 @@
       <c r="EA25" s="0">
         <v>124.314</v>
       </c>
+      <c r="EB25" s="0">
+        <v>125.381</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
@@ -8808,7 +8867,10 @@
         <v>124.407</v>
       </c>
       <c r="EA26" s="0">
-        <v>125.879</v>
+        <v>125.882</v>
+      </c>
+      <c r="EB26" s="0">
+        <v>128.014</v>
       </c>
     </row>
     <row r="27">
@@ -9203,7 +9265,10 @@
         <v>150.781</v>
       </c>
       <c r="EA27" s="4">
-        <v>152.23</v>
+        <v>152.306</v>
+      </c>
+      <c r="EB27" s="4">
+        <v>152.727</v>
       </c>
     </row>
     <row r="28">
@@ -9598,7 +9663,10 @@
         <v>151.644</v>
       </c>
       <c r="EA28" s="4">
-        <v>153.192</v>
+        <v>153.269</v>
+      </c>
+      <c r="EB28" s="4">
+        <v>153.617</v>
       </c>
     </row>
     <row r="29">
@@ -9993,7 +10061,10 @@
         <v>149.926</v>
       </c>
       <c r="EA29" s="0">
-        <v>151.963</v>
+        <v>151.974</v>
+      </c>
+      <c r="EB29" s="0">
+        <v>152.134</v>
       </c>
     </row>
     <row r="30">
@@ -10388,7 +10459,10 @@
         <v>153.676</v>
       </c>
       <c r="EA30" s="0">
-        <v>155.859</v>
+        <v>156.019</v>
+      </c>
+      <c r="EB30" s="0">
+        <v>155.939</v>
       </c>
     </row>
     <row r="31">
@@ -10783,7 +10857,10 @@
         <v>136.026</v>
       </c>
       <c r="EA31" s="0">
-        <v>137.574</v>
+        <v>137.117</v>
+      </c>
+      <c r="EB31" s="0">
+        <v>138.035</v>
       </c>
     </row>
     <row r="32">
@@ -11178,7 +11255,10 @@
         <v>152.983</v>
       </c>
       <c r="EA32" s="0">
-        <v>154.092</v>
+        <v>154.231</v>
+      </c>
+      <c r="EB32" s="0">
+        <v>154.742</v>
       </c>
     </row>
     <row r="33">
@@ -11573,7 +11653,10 @@
         <v>111.445</v>
       </c>
       <c r="EA33" s="4">
-        <v>108.879</v>
+        <v>108.885</v>
+      </c>
+      <c r="EB33" s="4">
+        <v>112.227</v>
       </c>
     </row>
     <row r="34">
@@ -11970,6 +12053,9 @@
       <c r="EA34" s="0" t="s">
         <v>5</v>
       </c>
+      <c r="EB34" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
@@ -12363,7 +12449,10 @@
         <v>144.456</v>
       </c>
       <c r="EA35" s="0">
-        <v>145.463</v>
+        <v>145.72</v>
+      </c>
+      <c r="EB35" s="0">
+        <v>145.791</v>
       </c>
     </row>
     <row r="36">
@@ -12758,7 +12847,10 @@
         <v>143.256</v>
       </c>
       <c r="EA36" s="0">
-        <v>144.398</v>
+        <v>144.684</v>
+      </c>
+      <c r="EB36" s="0">
+        <v>144.619</v>
       </c>
     </row>
     <row r="37">
@@ -13153,7 +13245,10 @@
         <v>136.122</v>
       </c>
       <c r="EA37" s="0">
-        <v>136.514</v>
+        <v>137.002</v>
+      </c>
+      <c r="EB37" s="0">
+        <v>136.741</v>
       </c>
     </row>
     <row r="38">
@@ -13548,7 +13643,10 @@
         <v>149.546</v>
       </c>
       <c r="EA38" s="0">
-        <v>151.401</v>
+        <v>151.493</v>
+      </c>
+      <c r="EB38" s="0">
+        <v>151.614</v>
       </c>
     </row>
     <row r="39">
@@ -13943,7 +14041,10 @@
         <v>94.587</v>
       </c>
       <c r="EA39" s="0">
-        <v>94.011</v>
+        <v>93.731</v>
+      </c>
+      <c r="EB39" s="0">
+        <v>92.23</v>
       </c>
     </row>
     <row r="40">
@@ -13998,10 +14099,10 @@
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A1:EA1"/>
-    <mergeCell ref="A2:EA2"/>
-    <mergeCell ref="A3:EA3"/>
-    <mergeCell ref="A4:EA4"/>
+    <mergeCell ref="A1:EB1"/>
+    <mergeCell ref="A2:EB2"/>
+    <mergeCell ref="A3:EB3"/>
+    <mergeCell ref="A4:EB4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:F6"/>
@@ -14036,16 +14137,17 @@
     <mergeCell ref="DO6:DR6"/>
     <mergeCell ref="DS6:DV6"/>
     <mergeCell ref="DW6:DZ6"/>
-    <mergeCell ref="A40:EB40"/>
-    <mergeCell ref="A41:EB41"/>
-    <mergeCell ref="A42:EB42"/>
-    <mergeCell ref="A43:EB43"/>
-    <mergeCell ref="A44:EB44"/>
-    <mergeCell ref="A45:EB45"/>
-    <mergeCell ref="A46:EB46"/>
-    <mergeCell ref="A47:EB47"/>
-    <mergeCell ref="A48:EB48"/>
-    <mergeCell ref="A49:EB49"/>
+    <mergeCell ref="EA6:EB6"/>
+    <mergeCell ref="A40:EC40"/>
+    <mergeCell ref="A41:EC41"/>
+    <mergeCell ref="A42:EC42"/>
+    <mergeCell ref="A43:EC43"/>
+    <mergeCell ref="A44:EC44"/>
+    <mergeCell ref="A45:EC45"/>
+    <mergeCell ref="A46:EC46"/>
+    <mergeCell ref="A47:EC47"/>
+    <mergeCell ref="A48:EC48"/>
+    <mergeCell ref="A49:EC49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BEA stats Jan 2026
</commit_message>
<xml_diff>
--- a/data/BEA/bea_const_price_indices.xlsx
+++ b/data/BEA/bea_const_price_indices.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="114">
   <si>
     <t xml:space="preserve">Table 5.3.4. Price Indexes for Private Fixed Investment by Type</t>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Bureau of Economic Analysis</t>
   </si>
   <si>
-    <t xml:space="preserve">Last Revised on: August 28, 2025 - Next Release Date September 25, 2025</t>
+    <t xml:space="preserve">Last Revised on: December 23, 2025 - Next Release Date January 22, 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Line</t>
@@ -555,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:EC49"/>
+  <dimension ref="A1:ED49"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.85" bestFit="1" customWidth="1" collapsed="1"/>
@@ -669,13 +669,13 @@
     <col min="109" max="109" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="110" max="110" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="111" max="111" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="112" max="112" width="7.800000000000001" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="112" max="112" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="113" max="113" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="114" max="114" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="115" max="115" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="116" max="116" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="117" max="117" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="118" max="118" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="118" max="118" width="7.800000000000001" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="119" max="119" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="120" max="120" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="121" max="121" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
@@ -690,6 +690,7 @@
     <col min="130" max="130" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="131" max="131" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="132" max="132" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="133" max="133" width="7.95" bestFit="1" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -916,6 +917,7 @@
         <v>38</v>
       </c>
       <c r="EB6" s="1"/>
+      <c r="EC6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="1"/>
@@ -1310,6 +1312,9 @@
       <c r="EB7" s="1" t="s">
         <v>40</v>
       </c>
+      <c r="EC7" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
@@ -1643,70 +1648,73 @@
         <v>103.15</v>
       </c>
       <c r="DG8" s="4">
-        <v>103.503</v>
+        <v>103.555</v>
       </c>
       <c r="DH8" s="4">
-        <v>103.869</v>
+        <v>103.913</v>
       </c>
       <c r="DI8" s="4">
-        <v>104.376</v>
+        <v>104.434</v>
       </c>
       <c r="DJ8" s="4">
-        <v>104.967</v>
+        <v>105.078</v>
       </c>
       <c r="DK8" s="4">
-        <v>105.689</v>
+        <v>105.811</v>
       </c>
       <c r="DL8" s="4">
-        <v>106.711</v>
+        <v>106.911</v>
       </c>
       <c r="DM8" s="4">
-        <v>108.537</v>
+        <v>108.643</v>
       </c>
       <c r="DN8" s="4">
-        <v>110.701</v>
+        <v>110.793</v>
       </c>
       <c r="DO8" s="4">
-        <v>113.302</v>
+        <v>113.264</v>
       </c>
       <c r="DP8" s="4">
-        <v>115.969</v>
+        <v>115.945</v>
       </c>
       <c r="DQ8" s="4">
-        <v>117.947</v>
+        <v>117.896</v>
       </c>
       <c r="DR8" s="4">
-        <v>119.06</v>
+        <v>118.923</v>
       </c>
       <c r="DS8" s="4">
-        <v>120.094</v>
+        <v>119.763</v>
       </c>
       <c r="DT8" s="4">
-        <v>120.055</v>
+        <v>119.636</v>
       </c>
       <c r="DU8" s="4">
-        <v>120.478</v>
+        <v>120.027</v>
       </c>
       <c r="DV8" s="4">
-        <v>121.164</v>
+        <v>120.719</v>
       </c>
       <c r="DW8" s="4">
-        <v>121.444</v>
+        <v>120.943</v>
       </c>
       <c r="DX8" s="4">
-        <v>122.22</v>
+        <v>121.751</v>
       </c>
       <c r="DY8" s="4">
-        <v>123.185</v>
+        <v>122.557</v>
       </c>
       <c r="DZ8" s="4">
-        <v>123.666</v>
+        <v>123.091</v>
       </c>
       <c r="EA8" s="4">
-        <v>124.042</v>
+        <v>123.316</v>
       </c>
       <c r="EB8" s="4">
-        <v>123.993</v>
+        <v>123.375</v>
+      </c>
+      <c r="EC8" s="4">
+        <v>124.916</v>
       </c>
     </row>
     <row r="9">
@@ -2041,70 +2049,73 @@
         <v>101.347</v>
       </c>
       <c r="DG9" s="4">
-        <v>101.62</v>
+        <v>101.623</v>
       </c>
       <c r="DH9" s="4">
-        <v>102.043</v>
+        <v>102.063</v>
       </c>
       <c r="DI9" s="4">
-        <v>101.977</v>
+        <v>101.994</v>
       </c>
       <c r="DJ9" s="4">
-        <v>102.172</v>
+        <v>102.2</v>
       </c>
       <c r="DK9" s="4">
-        <v>102.121</v>
+        <v>102.138</v>
       </c>
       <c r="DL9" s="4">
-        <v>102.198</v>
+        <v>102.246</v>
       </c>
       <c r="DM9" s="4">
-        <v>103.279</v>
+        <v>103.239</v>
       </c>
       <c r="DN9" s="4">
-        <v>104.982</v>
+        <v>104.965</v>
       </c>
       <c r="DO9" s="4">
-        <v>106.741</v>
+        <v>106.618</v>
       </c>
       <c r="DP9" s="4">
-        <v>108.815</v>
+        <v>108.739</v>
       </c>
       <c r="DQ9" s="4">
-        <v>110.544</v>
+        <v>110.547</v>
       </c>
       <c r="DR9" s="4">
-        <v>111.464</v>
+        <v>111.387</v>
       </c>
       <c r="DS9" s="4">
-        <v>112.979</v>
+        <v>112.712</v>
       </c>
       <c r="DT9" s="4">
-        <v>113.041</v>
+        <v>112.643</v>
       </c>
       <c r="DU9" s="4">
-        <v>113.169</v>
+        <v>112.662</v>
       </c>
       <c r="DV9" s="4">
-        <v>113.643</v>
+        <v>113.155</v>
       </c>
       <c r="DW9" s="4">
-        <v>114.02</v>
+        <v>113.378</v>
       </c>
       <c r="DX9" s="4">
-        <v>114.672</v>
+        <v>114.073</v>
       </c>
       <c r="DY9" s="4">
-        <v>115.554</v>
+        <v>114.705</v>
       </c>
       <c r="DZ9" s="4">
-        <v>115.98</v>
+        <v>115.141</v>
       </c>
       <c r="EA9" s="4">
-        <v>116.094</v>
+        <v>115.091</v>
       </c>
       <c r="EB9" s="4">
-        <v>115.943</v>
+        <v>114.985</v>
+      </c>
+      <c r="EC9" s="4">
+        <v>116.465</v>
       </c>
     </row>
     <row r="10">
@@ -2439,70 +2450,73 @@
         <v>106.603</v>
       </c>
       <c r="DG10" s="4">
-        <v>107.312</v>
+        <v>107.309</v>
       </c>
       <c r="DH10" s="4">
-        <v>106.869</v>
+        <v>106.936</v>
       </c>
       <c r="DI10" s="4">
-        <v>106.667</v>
+        <v>106.731</v>
       </c>
       <c r="DJ10" s="4">
-        <v>106.309</v>
+        <v>106.433</v>
       </c>
       <c r="DK10" s="4">
-        <v>106.435</v>
+        <v>106.484</v>
       </c>
       <c r="DL10" s="4">
-        <v>108.02</v>
+        <v>108.138</v>
       </c>
       <c r="DM10" s="4">
-        <v>110.377</v>
+        <v>110.468</v>
       </c>
       <c r="DN10" s="4">
-        <v>116.394</v>
+        <v>116.619</v>
       </c>
       <c r="DO10" s="4">
-        <v>121.105</v>
+        <v>121.339</v>
       </c>
       <c r="DP10" s="4">
-        <v>126.195</v>
+        <v>126.538</v>
       </c>
       <c r="DQ10" s="4">
-        <v>131.25</v>
+        <v>131.501</v>
       </c>
       <c r="DR10" s="4">
-        <v>133.821</v>
+        <v>134.11</v>
       </c>
       <c r="DS10" s="4">
-        <v>135.772</v>
+        <v>135.68</v>
       </c>
       <c r="DT10" s="4">
-        <v>135.408</v>
+        <v>135.325</v>
       </c>
       <c r="DU10" s="4">
-        <v>134.094</v>
+        <v>133.969</v>
       </c>
       <c r="DV10" s="4">
-        <v>135.21</v>
+        <v>135.138</v>
       </c>
       <c r="DW10" s="4">
-        <v>134.513</v>
+        <v>134.336</v>
       </c>
       <c r="DX10" s="4">
-        <v>134.625</v>
+        <v>134.935</v>
       </c>
       <c r="DY10" s="4">
-        <v>135.251</v>
+        <v>134.704</v>
       </c>
       <c r="DZ10" s="4">
-        <v>135.041</v>
+        <v>134.818</v>
       </c>
       <c r="EA10" s="4">
-        <v>135.879</v>
+        <v>135.174</v>
       </c>
       <c r="EB10" s="4">
-        <v>135.629</v>
+        <v>134.818</v>
+      </c>
+      <c r="EC10" s="4">
+        <v>136.022</v>
       </c>
     </row>
     <row r="11">
@@ -2837,70 +2851,73 @@
         <v>110.235</v>
       </c>
       <c r="DG11" s="0">
-        <v>110.967</v>
+        <v>110.851</v>
       </c>
       <c r="DH11" s="0">
         <v>110.97</v>
       </c>
       <c r="DI11" s="0">
-        <v>110.9</v>
+        <v>110.872</v>
       </c>
       <c r="DJ11" s="0">
-        <v>111.205</v>
+        <v>111.207</v>
       </c>
       <c r="DK11" s="0">
-        <v>111.941</v>
+        <v>111.69</v>
       </c>
       <c r="DL11" s="0">
-        <v>115.083</v>
+        <v>114.971</v>
       </c>
       <c r="DM11" s="0">
-        <v>118.08</v>
+        <v>117.946</v>
       </c>
       <c r="DN11" s="0">
-        <v>128.72</v>
+        <v>128.931</v>
       </c>
       <c r="DO11" s="0">
-        <v>135.667</v>
+        <v>135.627</v>
       </c>
       <c r="DP11" s="0">
-        <v>142.009</v>
+        <v>142.306</v>
       </c>
       <c r="DQ11" s="0">
-        <v>150.303</v>
+        <v>150.503</v>
       </c>
       <c r="DR11" s="0">
-        <v>154.708</v>
+        <v>155.032</v>
       </c>
       <c r="DS11" s="0">
-        <v>157.272</v>
+        <v>156.858</v>
       </c>
       <c r="DT11" s="0">
-        <v>157.032</v>
+        <v>156.923</v>
       </c>
       <c r="DU11" s="0">
-        <v>155.343</v>
+        <v>155.2</v>
       </c>
       <c r="DV11" s="0">
-        <v>154.985</v>
+        <v>155.038</v>
       </c>
       <c r="DW11" s="0">
-        <v>155.399</v>
+        <v>154.981</v>
       </c>
       <c r="DX11" s="0">
-        <v>155.632</v>
+        <v>155.628</v>
       </c>
       <c r="DY11" s="0">
-        <v>156.684</v>
+        <v>156.266</v>
       </c>
       <c r="DZ11" s="0">
-        <v>156.951</v>
+        <v>156.562</v>
       </c>
       <c r="EA11" s="0">
-        <v>158.351</v>
+        <v>157.179</v>
       </c>
       <c r="EB11" s="0">
-        <v>157.877</v>
+        <v>156.858</v>
+      </c>
+      <c r="EC11" s="0">
+        <v>157.55</v>
       </c>
     </row>
     <row r="12">
@@ -3235,70 +3252,73 @@
         <v>112.418</v>
       </c>
       <c r="DG12" s="0">
-        <v>113.132</v>
+        <v>113.058</v>
       </c>
       <c r="DH12" s="0">
-        <v>114.055</v>
+        <v>113.949</v>
       </c>
       <c r="DI12" s="0">
-        <v>114.832</v>
+        <v>114.63</v>
       </c>
       <c r="DJ12" s="0">
-        <v>114.625</v>
+        <v>114.655</v>
       </c>
       <c r="DK12" s="0">
-        <v>115.214</v>
+        <v>115.1</v>
       </c>
       <c r="DL12" s="0">
-        <v>116.114</v>
+        <v>116.025</v>
       </c>
       <c r="DM12" s="0">
-        <v>119.486</v>
+        <v>119.272</v>
       </c>
       <c r="DN12" s="0">
-        <v>129.616</v>
+        <v>129.688</v>
       </c>
       <c r="DO12" s="0">
-        <v>135.569</v>
+        <v>135.363</v>
       </c>
       <c r="DP12" s="0">
-        <v>142.808</v>
+        <v>142.732</v>
       </c>
       <c r="DQ12" s="0">
-        <v>152.314</v>
+        <v>152.052</v>
       </c>
       <c r="DR12" s="0">
-        <v>156.805</v>
+        <v>156.934</v>
       </c>
       <c r="DS12" s="0">
-        <v>159.33</v>
+        <v>158.993</v>
       </c>
       <c r="DT12" s="0">
-        <v>158.619</v>
+        <v>158.574</v>
       </c>
       <c r="DU12" s="0">
-        <v>156.7</v>
+        <v>156.45</v>
       </c>
       <c r="DV12" s="0">
-        <v>157.405</v>
+        <v>157.57</v>
       </c>
       <c r="DW12" s="0">
-        <v>157.684</v>
+        <v>157.266</v>
       </c>
       <c r="DX12" s="0">
-        <v>157.017</v>
+        <v>157.413</v>
       </c>
       <c r="DY12" s="0">
-        <v>157.342</v>
+        <v>157.525</v>
       </c>
       <c r="DZ12" s="0">
-        <v>156.648</v>
+        <v>157.263</v>
       </c>
       <c r="EA12" s="0">
-        <v>157.793</v>
+        <v>157.786</v>
       </c>
       <c r="EB12" s="0">
-        <v>158.166</v>
+        <v>158.131</v>
+      </c>
+      <c r="EC12" s="0">
+        <v>159.332</v>
       </c>
     </row>
     <row r="13">
@@ -3633,70 +3653,73 @@
         <v>104.218</v>
       </c>
       <c r="DG13" s="0">
-        <v>105.218</v>
+        <v>105.268</v>
       </c>
       <c r="DH13" s="0">
-        <v>105.487</v>
+        <v>105.579</v>
       </c>
       <c r="DI13" s="0">
-        <v>105.531</v>
+        <v>105.651</v>
       </c>
       <c r="DJ13" s="0">
-        <v>105.679</v>
+        <v>105.807</v>
       </c>
       <c r="DK13" s="0">
-        <v>106.131</v>
+        <v>106.252</v>
       </c>
       <c r="DL13" s="0">
-        <v>108.148</v>
+        <v>108.26</v>
       </c>
       <c r="DM13" s="0">
-        <v>110.851</v>
+        <v>110.955</v>
       </c>
       <c r="DN13" s="0">
-        <v>113.495</v>
+        <v>113.596</v>
       </c>
       <c r="DO13" s="0">
-        <v>115.985</v>
+        <v>116.075</v>
       </c>
       <c r="DP13" s="0">
-        <v>118.799</v>
+        <v>118.899</v>
       </c>
       <c r="DQ13" s="0">
-        <v>121.088</v>
+        <v>121.216</v>
       </c>
       <c r="DR13" s="0">
-        <v>122.254</v>
+        <v>122.421</v>
       </c>
       <c r="DS13" s="0">
-        <v>122.719</v>
+        <v>122.942</v>
       </c>
       <c r="DT13" s="0">
-        <v>123.246</v>
+        <v>123.381</v>
       </c>
       <c r="DU13" s="0">
-        <v>123.377</v>
+        <v>123.231</v>
       </c>
       <c r="DV13" s="0">
-        <v>123.535</v>
+        <v>123.038</v>
       </c>
       <c r="DW13" s="0">
-        <v>123.169</v>
+        <v>122.211</v>
       </c>
       <c r="DX13" s="0">
-        <v>122.534</v>
+        <v>121.191</v>
       </c>
       <c r="DY13" s="0">
-        <v>121.801</v>
+        <v>120.185</v>
       </c>
       <c r="DZ13" s="0">
-        <v>121.064</v>
+        <v>119.294</v>
       </c>
       <c r="EA13" s="0">
-        <v>120.692</v>
+        <v>118.955</v>
       </c>
       <c r="EB13" s="0">
-        <v>121.194</v>
+        <v>119.401</v>
+      </c>
+      <c r="EC13" s="0">
+        <v>119.638</v>
       </c>
     </row>
     <row r="14">
@@ -4031,70 +4054,73 @@
         <v>95.611</v>
       </c>
       <c r="DG14" s="0">
-        <v>95.845</v>
+        <v>96.006</v>
       </c>
       <c r="DH14" s="0">
-        <v>91.411</v>
+        <v>91.717</v>
       </c>
       <c r="DI14" s="0">
-        <v>87.991</v>
+        <v>88.433</v>
       </c>
       <c r="DJ14" s="0">
-        <v>83.686</v>
+        <v>84.259</v>
       </c>
       <c r="DK14" s="0">
-        <v>79.671</v>
+        <v>80.372</v>
       </c>
       <c r="DL14" s="0">
-        <v>77.863</v>
+        <v>78.616</v>
       </c>
       <c r="DM14" s="0">
-        <v>77.012</v>
+        <v>77.728</v>
       </c>
       <c r="DN14" s="0">
-        <v>77.972</v>
+        <v>78.54</v>
       </c>
       <c r="DO14" s="0">
-        <v>81.395</v>
+        <v>82.676</v>
       </c>
       <c r="DP14" s="0">
-        <v>86.669</v>
+        <v>87.832</v>
       </c>
       <c r="DQ14" s="0">
-        <v>87.438</v>
+        <v>88.432</v>
       </c>
       <c r="DR14" s="0">
-        <v>87.102</v>
+        <v>87.734</v>
       </c>
       <c r="DS14" s="0">
-        <v>90.948</v>
+        <v>91.176</v>
       </c>
       <c r="DT14" s="0">
-        <v>90.205</v>
+        <v>89.638</v>
       </c>
       <c r="DU14" s="0">
-        <v>87.061</v>
+        <v>86.615</v>
       </c>
       <c r="DV14" s="0">
-        <v>92.826</v>
+        <v>92.534</v>
       </c>
       <c r="DW14" s="0">
-        <v>88.832</v>
+        <v>89.318</v>
       </c>
       <c r="DX14" s="0">
-        <v>89.978</v>
+        <v>92.162</v>
       </c>
       <c r="DY14" s="0">
-        <v>91.185</v>
+        <v>89.352</v>
       </c>
       <c r="DZ14" s="0">
-        <v>90.835</v>
+        <v>90.548</v>
       </c>
       <c r="EA14" s="0">
-        <v>91.544</v>
+        <v>90.221</v>
       </c>
       <c r="EB14" s="0">
-        <v>89.036</v>
+        <v>86.808</v>
+      </c>
+      <c r="EC14" s="0">
+        <v>90.697</v>
       </c>
     </row>
     <row r="15">
@@ -4429,70 +4455,73 @@
         <v>110.235</v>
       </c>
       <c r="DG15" s="0">
-        <v>111.323</v>
+        <v>111.328</v>
       </c>
       <c r="DH15" s="0">
-        <v>111.718</v>
+        <v>111.737</v>
       </c>
       <c r="DI15" s="0">
-        <v>112.309</v>
+        <v>112.305</v>
       </c>
       <c r="DJ15" s="0">
         <v>112.669</v>
       </c>
       <c r="DK15" s="0">
-        <v>114.237</v>
+        <v>114.243</v>
       </c>
       <c r="DL15" s="0">
-        <v>115.964</v>
+        <v>115.994</v>
       </c>
       <c r="DM15" s="0">
-        <v>119.074</v>
+        <v>119.067</v>
       </c>
       <c r="DN15" s="0">
-        <v>122.525</v>
+        <v>122.509</v>
       </c>
       <c r="DO15" s="0">
-        <v>125.888</v>
+        <v>125.865</v>
       </c>
       <c r="DP15" s="0">
-        <v>129.26</v>
+        <v>129.271</v>
       </c>
       <c r="DQ15" s="0">
-        <v>132.434</v>
+        <v>132.374</v>
       </c>
       <c r="DR15" s="0">
-        <v>134.807</v>
+        <v>134.754</v>
       </c>
       <c r="DS15" s="0">
-        <v>134.859</v>
+        <v>134.813</v>
       </c>
       <c r="DT15" s="0">
-        <v>134.274</v>
+        <v>134.314</v>
       </c>
       <c r="DU15" s="0">
-        <v>134.595</v>
+        <v>134.593</v>
       </c>
       <c r="DV15" s="0">
-        <v>135.122</v>
+        <v>135.185</v>
       </c>
       <c r="DW15" s="0">
-        <v>134.319</v>
+        <v>134.658</v>
       </c>
       <c r="DX15" s="0">
-        <v>135.013</v>
+        <v>135.473</v>
       </c>
       <c r="DY15" s="0">
-        <v>136.314</v>
+        <v>136.672</v>
       </c>
       <c r="DZ15" s="0">
-        <v>136.7</v>
+        <v>137.154</v>
       </c>
       <c r="EA15" s="0">
-        <v>137.817</v>
+        <v>138.387</v>
       </c>
       <c r="EB15" s="0">
-        <v>138.144</v>
+        <v>138.727</v>
+      </c>
+      <c r="EC15" s="0">
+        <v>139.763</v>
       </c>
     </row>
     <row r="16">
@@ -4827,70 +4856,73 @@
         <v>99.591</v>
       </c>
       <c r="DG16" s="4">
-        <v>99.648</v>
+        <v>99.651</v>
       </c>
       <c r="DH16" s="4">
-        <v>99.812</v>
+        <v>99.819</v>
       </c>
       <c r="DI16" s="4">
-        <v>99.482</v>
+        <v>99.488</v>
       </c>
       <c r="DJ16" s="4">
-        <v>98.871</v>
+        <v>98.886</v>
       </c>
       <c r="DK16" s="4">
-        <v>99.444</v>
+        <v>99.474</v>
       </c>
       <c r="DL16" s="4">
-        <v>98.72</v>
+        <v>98.749</v>
       </c>
       <c r="DM16" s="4">
-        <v>99.993</v>
+        <v>100.058</v>
       </c>
       <c r="DN16" s="4">
-        <v>101.29</v>
+        <v>101.351</v>
       </c>
       <c r="DO16" s="4">
-        <v>103.189</v>
+        <v>103.206</v>
       </c>
       <c r="DP16" s="4">
-        <v>105.425</v>
+        <v>105.439</v>
       </c>
       <c r="DQ16" s="4">
-        <v>107.073</v>
+        <v>107.049</v>
       </c>
       <c r="DR16" s="4">
-        <v>108.629</v>
+        <v>108.567</v>
       </c>
       <c r="DS16" s="4">
-        <v>110.488</v>
+        <v>110.39</v>
       </c>
       <c r="DT16" s="4">
-        <v>110.531</v>
+        <v>110.463</v>
       </c>
       <c r="DU16" s="4">
-        <v>111.218</v>
+        <v>111.162</v>
       </c>
       <c r="DV16" s="4">
-        <v>111.531</v>
+        <v>111.444</v>
       </c>
       <c r="DW16" s="4">
-        <v>112.583</v>
+        <v>112.427</v>
       </c>
       <c r="DX16" s="4">
-        <v>113.057</v>
+        <v>112.956</v>
       </c>
       <c r="DY16" s="4">
-        <v>113.744</v>
+        <v>113.547</v>
       </c>
       <c r="DZ16" s="4">
-        <v>114.017</v>
+        <v>113.761</v>
       </c>
       <c r="EA16" s="4">
-        <v>114.23</v>
+        <v>113.939</v>
       </c>
       <c r="EB16" s="4">
-        <v>115.028</v>
+        <v>114.879</v>
+      </c>
+      <c r="EC16" s="4">
+        <v>116.505</v>
       </c>
     </row>
     <row r="17">
@@ -5225,70 +5257,73 @@
         <v>93.22</v>
       </c>
       <c r="DG17" s="0">
-        <v>92.904</v>
+        <v>92.91</v>
       </c>
       <c r="DH17" s="0">
-        <v>92.565</v>
+        <v>92.567</v>
       </c>
       <c r="DI17" s="0">
-        <v>92.544</v>
+        <v>92.548</v>
       </c>
       <c r="DJ17" s="0">
-        <v>92.259</v>
+        <v>92.261</v>
       </c>
       <c r="DK17" s="0">
-        <v>92.274</v>
+        <v>92.267</v>
       </c>
       <c r="DL17" s="0">
-        <v>92.239</v>
+        <v>92.238</v>
       </c>
       <c r="DM17" s="0">
-        <v>92.439</v>
+        <v>92.441</v>
       </c>
       <c r="DN17" s="0">
-        <v>92.454</v>
+        <v>92.455</v>
       </c>
       <c r="DO17" s="0">
-        <v>93.625</v>
+        <v>93.614</v>
       </c>
       <c r="DP17" s="0">
-        <v>93.888</v>
+        <v>93.877</v>
       </c>
       <c r="DQ17" s="0">
-        <v>93.948</v>
+        <v>93.933</v>
       </c>
       <c r="DR17" s="0">
-        <v>94.271</v>
+        <v>94.254</v>
       </c>
       <c r="DS17" s="0">
-        <v>95.182</v>
+        <v>95.147</v>
       </c>
       <c r="DT17" s="0">
-        <v>95.335</v>
+        <v>95.347</v>
       </c>
       <c r="DU17" s="0">
-        <v>95.416</v>
+        <v>95.385</v>
       </c>
       <c r="DV17" s="0">
-        <v>95.509</v>
+        <v>95.455</v>
       </c>
       <c r="DW17" s="0">
-        <v>96.366</v>
+        <v>96.281</v>
       </c>
       <c r="DX17" s="0">
-        <v>96.76</v>
+        <v>96.658</v>
       </c>
       <c r="DY17" s="0">
-        <v>97.2</v>
+        <v>97.095</v>
       </c>
       <c r="DZ17" s="0">
-        <v>97.603</v>
+        <v>97.483</v>
       </c>
       <c r="EA17" s="0">
-        <v>97.918</v>
+        <v>97.741</v>
       </c>
       <c r="EB17" s="0">
-        <v>98.33</v>
+        <v>98.542</v>
+      </c>
+      <c r="EC17" s="0">
+        <v>100.231</v>
       </c>
     </row>
     <row r="18">
@@ -5623,70 +5658,73 @@
         <v>96.404</v>
       </c>
       <c r="DG18" s="0">
-        <v>96.042</v>
+        <v>96.071</v>
       </c>
       <c r="DH18" s="0">
         <v>96.364</v>
       </c>
       <c r="DI18" s="0">
-        <v>96.454</v>
+        <v>96.466</v>
       </c>
       <c r="DJ18" s="0">
         <v>96.206</v>
       </c>
       <c r="DK18" s="0">
-        <v>96.805</v>
+        <v>96.793</v>
       </c>
       <c r="DL18" s="0">
-        <v>97.239</v>
+        <v>97.244</v>
       </c>
       <c r="DM18" s="0">
-        <v>98.275</v>
+        <v>98.28</v>
       </c>
       <c r="DN18" s="0">
-        <v>98.769</v>
+        <v>98.787</v>
       </c>
       <c r="DO18" s="0">
-        <v>100.732</v>
+        <v>100.721</v>
       </c>
       <c r="DP18" s="0">
-        <v>101.473</v>
+        <v>101.47</v>
       </c>
       <c r="DQ18" s="0">
-        <v>101.397</v>
+        <v>101.44</v>
       </c>
       <c r="DR18" s="0">
-        <v>102.049</v>
+        <v>102.083</v>
       </c>
       <c r="DS18" s="0">
-        <v>102.692</v>
+        <v>102.668</v>
       </c>
       <c r="DT18" s="0">
-        <v>101.641</v>
+        <v>101.662</v>
       </c>
       <c r="DU18" s="0">
-        <v>101.377</v>
+        <v>101.362</v>
       </c>
       <c r="DV18" s="0">
-        <v>101.6</v>
+        <v>101.558</v>
       </c>
       <c r="DW18" s="0">
-        <v>102.066</v>
+        <v>101.986</v>
       </c>
       <c r="DX18" s="0">
-        <v>102.174</v>
+        <v>102.061</v>
       </c>
       <c r="DY18" s="0">
-        <v>102.113</v>
+        <v>101.98</v>
       </c>
       <c r="DZ18" s="0">
-        <v>102.603</v>
+        <v>102.426</v>
       </c>
       <c r="EA18" s="0">
-        <v>102.902</v>
+        <v>102.65</v>
       </c>
       <c r="EB18" s="0">
-        <v>102.799</v>
+        <v>103.678</v>
+      </c>
+      <c r="EC18" s="0">
+        <v>104.293</v>
       </c>
     </row>
     <row r="19">
@@ -6027,64 +6065,67 @@
         <v>91.073</v>
       </c>
       <c r="DI19" s="0">
-        <v>91.006</v>
+        <v>91.007</v>
       </c>
       <c r="DJ19" s="0">
-        <v>90.709</v>
+        <v>90.711</v>
       </c>
       <c r="DK19" s="0">
-        <v>90.454</v>
+        <v>90.453</v>
       </c>
       <c r="DL19" s="0">
-        <v>90.205</v>
+        <v>90.206</v>
       </c>
       <c r="DM19" s="0">
         <v>90.028</v>
       </c>
       <c r="DN19" s="0">
-        <v>89.822</v>
+        <v>89.813</v>
       </c>
       <c r="DO19" s="0">
-        <v>90.63</v>
+        <v>90.62</v>
       </c>
       <c r="DP19" s="0">
-        <v>90.679</v>
+        <v>90.666</v>
       </c>
       <c r="DQ19" s="0">
-        <v>90.803</v>
+        <v>90.766</v>
       </c>
       <c r="DR19" s="0">
-        <v>90.986</v>
+        <v>90.95</v>
       </c>
       <c r="DS19" s="0">
-        <v>92.022</v>
+        <v>91.986</v>
       </c>
       <c r="DT19" s="0">
-        <v>92.695</v>
+        <v>92.7</v>
       </c>
       <c r="DU19" s="0">
-        <v>92.929</v>
+        <v>92.886</v>
       </c>
       <c r="DV19" s="0">
-        <v>92.967</v>
+        <v>92.905</v>
       </c>
       <c r="DW19" s="0">
-        <v>94.012</v>
+        <v>93.916</v>
       </c>
       <c r="DX19" s="0">
-        <v>94.551</v>
+        <v>94.445</v>
       </c>
       <c r="DY19" s="0">
-        <v>95.259</v>
+        <v>95.157</v>
       </c>
       <c r="DZ19" s="0">
-        <v>95.619</v>
+        <v>95.515</v>
       </c>
       <c r="EA19" s="0">
-        <v>95.945</v>
+        <v>95.794</v>
       </c>
       <c r="EB19" s="0">
-        <v>96.68</v>
+        <v>96.464</v>
+      </c>
+      <c r="EC19" s="0">
+        <v>98.949</v>
       </c>
     </row>
     <row r="20">
@@ -6419,70 +6460,73 @@
         <v>103.916</v>
       </c>
       <c r="DG20" s="0">
-        <v>104.261</v>
+        <v>104.263</v>
       </c>
       <c r="DH20" s="0">
-        <v>104.182</v>
+        <v>104.185</v>
       </c>
       <c r="DI20" s="0">
-        <v>104.475</v>
+        <v>104.481</v>
       </c>
       <c r="DJ20" s="0">
-        <v>104.91</v>
+        <v>104.917</v>
       </c>
       <c r="DK20" s="0">
-        <v>106.09</v>
+        <v>106.094</v>
       </c>
       <c r="DL20" s="0">
-        <v>107.876</v>
+        <v>107.891</v>
       </c>
       <c r="DM20" s="0">
-        <v>109.949</v>
+        <v>109.978</v>
       </c>
       <c r="DN20" s="0">
-        <v>111.851</v>
+        <v>111.891</v>
       </c>
       <c r="DO20" s="0">
-        <v>114.911</v>
+        <v>114.968</v>
       </c>
       <c r="DP20" s="0">
-        <v>117.514</v>
+        <v>117.557</v>
       </c>
       <c r="DQ20" s="0">
-        <v>118.888</v>
+        <v>118.924</v>
       </c>
       <c r="DR20" s="0">
-        <v>119.564</v>
+        <v>119.54</v>
       </c>
       <c r="DS20" s="0">
-        <v>121.354</v>
+        <v>121.326</v>
       </c>
       <c r="DT20" s="0">
-        <v>122.192</v>
+        <v>122.147</v>
       </c>
       <c r="DU20" s="0">
-        <v>122.752</v>
+        <v>122.702</v>
       </c>
       <c r="DV20" s="0">
-        <v>122.934</v>
+        <v>122.881</v>
       </c>
       <c r="DW20" s="0">
-        <v>124.21</v>
+        <v>124.131</v>
       </c>
       <c r="DX20" s="0">
-        <v>125.212</v>
+        <v>125.027</v>
       </c>
       <c r="DY20" s="0">
-        <v>125.737</v>
+        <v>125.525</v>
       </c>
       <c r="DZ20" s="0">
-        <v>126.089</v>
+        <v>125.868</v>
       </c>
       <c r="EA20" s="0">
-        <v>127.022</v>
+        <v>126.831</v>
       </c>
       <c r="EB20" s="0">
-        <v>128.438</v>
+        <v>128.22</v>
+      </c>
+      <c r="EC20" s="0">
+        <v>130.798</v>
       </c>
     </row>
     <row r="21">
@@ -6817,70 +6861,73 @@
         <v>100.83</v>
       </c>
       <c r="DG21" s="0">
-        <v>101.174</v>
+        <v>101.179</v>
       </c>
       <c r="DH21" s="0">
-        <v>102.604</v>
+        <v>102.625</v>
       </c>
       <c r="DI21" s="0">
-        <v>100.462</v>
+        <v>100.445</v>
       </c>
       <c r="DJ21" s="0">
-        <v>97.512</v>
+        <v>97.49</v>
       </c>
       <c r="DK21" s="0">
-        <v>98.906</v>
+        <v>98.902</v>
       </c>
       <c r="DL21" s="0">
-        <v>91.957</v>
+        <v>91.842</v>
       </c>
       <c r="DM21" s="0">
-        <v>93.473</v>
+        <v>93.447</v>
       </c>
       <c r="DN21" s="0">
-        <v>94.619</v>
+        <v>94.52</v>
       </c>
       <c r="DO21" s="0">
-        <v>94.835</v>
+        <v>94.516</v>
       </c>
       <c r="DP21" s="0">
-        <v>99.436</v>
+        <v>99.082</v>
       </c>
       <c r="DQ21" s="0">
-        <v>102.732</v>
+        <v>102.315</v>
       </c>
       <c r="DR21" s="0">
-        <v>107.195</v>
+        <v>106.662</v>
       </c>
       <c r="DS21" s="0">
-        <v>111.024</v>
+        <v>110.426</v>
       </c>
       <c r="DT21" s="0">
-        <v>109.422</v>
+        <v>108.866</v>
       </c>
       <c r="DU21" s="0">
-        <v>111.045</v>
+        <v>110.605</v>
       </c>
       <c r="DV21" s="0">
-        <v>111.904</v>
+        <v>111.444</v>
       </c>
       <c r="DW21" s="0">
-        <v>113.273</v>
+        <v>112.677</v>
       </c>
       <c r="DX21" s="0">
-        <v>113.326</v>
+        <v>113.103</v>
       </c>
       <c r="DY21" s="0">
-        <v>114.782</v>
+        <v>114.23</v>
       </c>
       <c r="DZ21" s="0">
-        <v>114.777</v>
+        <v>113.997</v>
       </c>
       <c r="EA21" s="0">
-        <v>114.106</v>
+        <v>113.21</v>
       </c>
       <c r="EB21" s="0">
-        <v>114.821</v>
+        <v>113.845</v>
+      </c>
+      <c r="EC21" s="0">
+        <v>113.78</v>
       </c>
     </row>
     <row r="22">
@@ -7215,70 +7262,73 @@
         <v>104.49</v>
       </c>
       <c r="DG22" s="0">
-        <v>104.707</v>
+        <v>104.701</v>
       </c>
       <c r="DH22" s="0">
-        <v>104.907</v>
+        <v>104.914</v>
       </c>
       <c r="DI22" s="0">
-        <v>104.93</v>
+        <v>104.948</v>
       </c>
       <c r="DJ22" s="0">
-        <v>104.807</v>
+        <v>104.841</v>
       </c>
       <c r="DK22" s="0">
-        <v>104.947</v>
+        <v>105.055</v>
       </c>
       <c r="DL22" s="0">
-        <v>106.531</v>
+        <v>106.661</v>
       </c>
       <c r="DM22" s="0">
-        <v>108.72</v>
+        <v>108.913</v>
       </c>
       <c r="DN22" s="0">
-        <v>111.994</v>
+        <v>112.2</v>
       </c>
       <c r="DO22" s="0">
-        <v>115.506</v>
+        <v>115.682</v>
       </c>
       <c r="DP22" s="0">
-        <v>119.367</v>
+        <v>119.543</v>
       </c>
       <c r="DQ22" s="0">
-        <v>122.95</v>
+        <v>123.021</v>
       </c>
       <c r="DR22" s="0">
-        <v>124.931</v>
+        <v>125</v>
       </c>
       <c r="DS22" s="0">
-        <v>126.527</v>
+        <v>126.521</v>
       </c>
       <c r="DT22" s="0">
-        <v>127.27</v>
+        <v>127.305</v>
       </c>
       <c r="DU22" s="0">
-        <v>128.045</v>
+        <v>128.13</v>
       </c>
       <c r="DV22" s="0">
-        <v>128.233</v>
+        <v>128.279</v>
       </c>
       <c r="DW22" s="0">
-        <v>129.058</v>
+        <v>129.05</v>
       </c>
       <c r="DX22" s="0">
-        <v>129.625</v>
+        <v>129.659</v>
       </c>
       <c r="DY22" s="0">
-        <v>130.002</v>
+        <v>130.016</v>
       </c>
       <c r="DZ22" s="0">
-        <v>130.255</v>
+        <v>130.283</v>
       </c>
       <c r="EA22" s="0">
-        <v>130.583</v>
+        <v>130.633</v>
       </c>
       <c r="EB22" s="0">
-        <v>131.708</v>
+        <v>131.736</v>
+      </c>
+      <c r="EC22" s="0">
+        <v>134.239</v>
       </c>
     </row>
     <row r="23">
@@ -7613,70 +7663,73 @@
         <v>100.251</v>
       </c>
       <c r="DG23" s="4">
-        <v>100.559</v>
+        <v>100.565</v>
       </c>
       <c r="DH23" s="4">
-        <v>101.739</v>
+        <v>101.746</v>
       </c>
       <c r="DI23" s="4">
-        <v>102.004</v>
+        <v>102.008</v>
       </c>
       <c r="DJ23" s="4">
-        <v>103.276</v>
+        <v>103.269</v>
       </c>
       <c r="DK23" s="4">
-        <v>102.46</v>
+        <v>102.443</v>
       </c>
       <c r="DL23" s="4">
-        <v>102.573</v>
+        <v>102.607</v>
       </c>
       <c r="DM23" s="4">
-        <v>102.833</v>
+        <v>102.629</v>
       </c>
       <c r="DN23" s="4">
-        <v>102.953</v>
+        <v>102.755</v>
       </c>
       <c r="DO23" s="4">
-        <v>103.271</v>
+        <v>102.875</v>
       </c>
       <c r="DP23" s="4">
-        <v>103.868</v>
+        <v>103.553</v>
       </c>
       <c r="DQ23" s="4">
-        <v>104.215</v>
+        <v>104.163</v>
       </c>
       <c r="DR23" s="4">
-        <v>103.834</v>
+        <v>103.614</v>
       </c>
       <c r="DS23" s="4">
-        <v>104.833</v>
+        <v>104.366</v>
       </c>
       <c r="DT23" s="4">
-        <v>105.091</v>
+        <v>104.281</v>
       </c>
       <c r="DU23" s="4">
-        <v>105.368</v>
+        <v>104.34</v>
       </c>
       <c r="DV23" s="4">
-        <v>105.686</v>
+        <v>104.689</v>
       </c>
       <c r="DW23" s="4">
-        <v>105.962</v>
+        <v>104.751</v>
       </c>
       <c r="DX23" s="4">
-        <v>107.016</v>
+        <v>105.638</v>
       </c>
       <c r="DY23" s="4">
-        <v>108.186</v>
+        <v>106.706</v>
       </c>
       <c r="DZ23" s="4">
-        <v>109.033</v>
+        <v>107.482</v>
       </c>
       <c r="EA23" s="4">
-        <v>108.735</v>
+        <v>107.051</v>
       </c>
       <c r="EB23" s="4">
-        <v>107.763</v>
+        <v>106.117</v>
+      </c>
+      <c r="EC23" s="4">
+        <v>107.569</v>
       </c>
     </row>
     <row r="24">
@@ -8011,70 +8064,73 @@
         <v>94.778</v>
       </c>
       <c r="DG24" s="0">
-        <v>94.026</v>
+        <v>94.037</v>
       </c>
       <c r="DH24" s="0">
-        <v>93.854</v>
+        <v>93.866</v>
       </c>
       <c r="DI24" s="0">
-        <v>93.34</v>
+        <v>93.341</v>
       </c>
       <c r="DJ24" s="0">
-        <v>93.361</v>
+        <v>93.342</v>
       </c>
       <c r="DK24" s="0">
-        <v>91.259</v>
+        <v>91.21</v>
       </c>
       <c r="DL24" s="0">
-        <v>91.198</v>
+        <v>91.111</v>
       </c>
       <c r="DM24" s="0">
-        <v>90.839</v>
+        <v>90.711</v>
       </c>
       <c r="DN24" s="0">
-        <v>90.535</v>
+        <v>90.358</v>
       </c>
       <c r="DO24" s="0">
-        <v>89.482</v>
+        <v>89.255</v>
       </c>
       <c r="DP24" s="0">
-        <v>89.539</v>
+        <v>89.286</v>
       </c>
       <c r="DQ24" s="0">
-        <v>89.865</v>
+        <v>89.614</v>
       </c>
       <c r="DR24" s="0">
-        <v>88.49</v>
+        <v>88.272</v>
       </c>
       <c r="DS24" s="0">
-        <v>89.989</v>
+        <v>89.823</v>
       </c>
       <c r="DT24" s="0">
-        <v>89.443</v>
+        <v>89.251</v>
       </c>
       <c r="DU24" s="0">
-        <v>89.199</v>
+        <v>88.901</v>
       </c>
       <c r="DV24" s="0">
-        <v>89.047</v>
+        <v>88.567</v>
       </c>
       <c r="DW24" s="0">
-        <v>88.732</v>
+        <v>87.993</v>
       </c>
       <c r="DX24" s="0">
-        <v>90.245</v>
+        <v>89.295</v>
       </c>
       <c r="DY24" s="0">
-        <v>91.858</v>
+        <v>90.752</v>
       </c>
       <c r="DZ24" s="0">
-        <v>92.241</v>
+        <v>91.063</v>
       </c>
       <c r="EA24" s="0">
-        <v>90.559</v>
+        <v>89.168</v>
       </c>
       <c r="EB24" s="0">
-        <v>87.662</v>
+        <v>86.369</v>
+      </c>
+      <c r="EC24" s="0">
+        <v>87.974</v>
       </c>
     </row>
     <row r="25">
@@ -8409,70 +8465,73 @@
         <v>104.781</v>
       </c>
       <c r="DG25" s="0">
-        <v>106.04</v>
+        <v>106.043</v>
       </c>
       <c r="DH25" s="0">
-        <v>108.479</v>
+        <v>108.483</v>
       </c>
       <c r="DI25" s="0">
-        <v>109.821</v>
+        <v>109.824</v>
       </c>
       <c r="DJ25" s="0">
-        <v>112.441</v>
+        <v>112.442</v>
       </c>
       <c r="DK25" s="0">
-        <v>112.617</v>
+        <v>112.627</v>
       </c>
       <c r="DL25" s="0">
-        <v>112.742</v>
+        <v>112.899</v>
       </c>
       <c r="DM25" s="0">
-        <v>113.467</v>
+        <v>113.144</v>
       </c>
       <c r="DN25" s="0">
-        <v>113.903</v>
+        <v>113.645</v>
       </c>
       <c r="DO25" s="0">
-        <v>115.445</v>
+        <v>114.797</v>
       </c>
       <c r="DP25" s="0">
-        <v>116.341</v>
+        <v>115.896</v>
       </c>
       <c r="DQ25" s="0">
-        <v>116.577</v>
+        <v>116.713</v>
       </c>
       <c r="DR25" s="0">
-        <v>117.092</v>
+        <v>116.812</v>
       </c>
       <c r="DS25" s="0">
-        <v>117.37</v>
+        <v>116.488</v>
       </c>
       <c r="DT25" s="0">
-        <v>118.276</v>
+        <v>116.654</v>
       </c>
       <c r="DU25" s="0">
-        <v>119.214</v>
+        <v>117.218</v>
       </c>
       <c r="DV25" s="0">
-        <v>119.797</v>
+        <v>118.079</v>
       </c>
       <c r="DW25" s="0">
-        <v>120.441</v>
+        <v>118.548</v>
       </c>
       <c r="DX25" s="0">
+        <v>119.024</v>
+      </c>
+      <c r="DY25" s="0">
+        <v>119.695</v>
+      </c>
+      <c r="DZ25" s="0">
         <v>121.046</v>
       </c>
-      <c r="DY25" s="0">
-        <v>121.764</v>
-      </c>
-      <c r="DZ25" s="0">
-        <v>123.186</v>
-      </c>
       <c r="EA25" s="0">
-        <v>124.314</v>
+        <v>122.128</v>
       </c>
       <c r="EB25" s="0">
-        <v>125.381</v>
+        <v>123.165</v>
+      </c>
+      <c r="EC25" s="0">
+        <v>124.455</v>
       </c>
     </row>
     <row r="26">
@@ -8840,7 +8899,7 @@
         <v>114.073</v>
       </c>
       <c r="DR26" s="0">
-        <v>115.131</v>
+        <v>115.13</v>
       </c>
       <c r="DS26" s="0">
         <v>117.135</v>
@@ -8849,28 +8908,31 @@
         <v>119.038</v>
       </c>
       <c r="DU26" s="0">
-        <v>118.713</v>
+        <v>118.715</v>
       </c>
       <c r="DV26" s="0">
-        <v>120.841</v>
+        <v>120.844</v>
       </c>
       <c r="DW26" s="0">
-        <v>123.268</v>
+        <v>123.232</v>
       </c>
       <c r="DX26" s="0">
-        <v>123.52</v>
+        <v>123.526</v>
       </c>
       <c r="DY26" s="0">
-        <v>124.006</v>
+        <v>124.017</v>
       </c>
       <c r="DZ26" s="0">
-        <v>124.407</v>
+        <v>124.424</v>
       </c>
       <c r="EA26" s="0">
-        <v>125.882</v>
+        <v>125.903</v>
       </c>
       <c r="EB26" s="0">
-        <v>128.014</v>
+        <v>128.03</v>
+      </c>
+      <c r="EC26" s="0">
+        <v>128.69</v>
       </c>
     </row>
     <row r="27">
@@ -9205,70 +9267,73 @@
         <v>109.736</v>
       </c>
       <c r="DG27" s="4">
-        <v>110.378</v>
+        <v>110.618</v>
       </c>
       <c r="DH27" s="4">
-        <v>110.553</v>
+        <v>110.689</v>
       </c>
       <c r="DI27" s="4">
-        <v>113.086</v>
+        <v>113.301</v>
       </c>
       <c r="DJ27" s="4">
-        <v>115.022</v>
+        <v>115.43</v>
       </c>
       <c r="DK27" s="4">
-        <v>118.282</v>
+        <v>118.783</v>
       </c>
       <c r="DL27" s="4">
-        <v>122.449</v>
+        <v>123.213</v>
       </c>
       <c r="DM27" s="4">
-        <v>126.817</v>
+        <v>127.499</v>
       </c>
       <c r="DN27" s="4">
-        <v>130.601</v>
+        <v>131.151</v>
       </c>
       <c r="DO27" s="4">
-        <v>136.158</v>
+        <v>136.505</v>
       </c>
       <c r="DP27" s="4">
-        <v>140.999</v>
+        <v>141.252</v>
       </c>
       <c r="DQ27" s="4">
-        <v>143.964</v>
+        <v>143.774</v>
       </c>
       <c r="DR27" s="4">
-        <v>145.894</v>
+        <v>145.583</v>
       </c>
       <c r="DS27" s="4">
-        <v>144.81</v>
+        <v>144.286</v>
       </c>
       <c r="DT27" s="4">
-        <v>144.359</v>
+        <v>143.922</v>
       </c>
       <c r="DU27" s="4">
-        <v>146.086</v>
+        <v>145.957</v>
       </c>
       <c r="DV27" s="4">
-        <v>147.689</v>
+        <v>147.496</v>
       </c>
       <c r="DW27" s="4">
-        <v>147.527</v>
+        <v>147.707</v>
       </c>
       <c r="DX27" s="4">
-        <v>148.802</v>
+        <v>148.968</v>
       </c>
       <c r="DY27" s="4">
-        <v>150.081</v>
+        <v>150.504</v>
       </c>
       <c r="DZ27" s="4">
-        <v>150.781</v>
+        <v>151.442</v>
       </c>
       <c r="EA27" s="4">
-        <v>152.306</v>
+        <v>152.891</v>
       </c>
       <c r="EB27" s="4">
-        <v>152.727</v>
+        <v>153.712</v>
+      </c>
+      <c r="EC27" s="4">
+        <v>155.426</v>
       </c>
     </row>
     <row r="28">
@@ -9603,70 +9668,73 @@
         <v>109.896</v>
       </c>
       <c r="DG28" s="4">
-        <v>110.536</v>
+        <v>110.777</v>
       </c>
       <c r="DH28" s="4">
-        <v>110.669</v>
+        <v>110.811</v>
       </c>
       <c r="DI28" s="4">
-        <v>113.15</v>
+        <v>113.373</v>
       </c>
       <c r="DJ28" s="4">
-        <v>115.047</v>
+        <v>115.463</v>
       </c>
       <c r="DK28" s="4">
-        <v>118.384</v>
+        <v>118.892</v>
       </c>
       <c r="DL28" s="4">
-        <v>122.587</v>
+        <v>123.368</v>
       </c>
       <c r="DM28" s="4">
-        <v>126.967</v>
+        <v>127.667</v>
       </c>
       <c r="DN28" s="4">
-        <v>130.78</v>
+        <v>131.341</v>
       </c>
       <c r="DO28" s="4">
-        <v>136.375</v>
+        <v>136.726</v>
       </c>
       <c r="DP28" s="4">
-        <v>141.284</v>
+        <v>141.541</v>
       </c>
       <c r="DQ28" s="4">
-        <v>144.361</v>
+        <v>144.173</v>
       </c>
       <c r="DR28" s="4">
-        <v>146.347</v>
+        <v>146.031</v>
       </c>
       <c r="DS28" s="4">
-        <v>145.291</v>
+        <v>144.752</v>
       </c>
       <c r="DT28" s="4">
-        <v>144.915</v>
+        <v>144.463</v>
       </c>
       <c r="DU28" s="4">
-        <v>146.73</v>
+        <v>146.604</v>
       </c>
       <c r="DV28" s="4">
-        <v>148.425</v>
+        <v>148.229</v>
       </c>
       <c r="DW28" s="4">
-        <v>148.239</v>
+        <v>148.421</v>
       </c>
       <c r="DX28" s="4">
-        <v>149.604</v>
+        <v>149.767</v>
       </c>
       <c r="DY28" s="4">
-        <v>150.902</v>
+        <v>151.342</v>
       </c>
       <c r="DZ28" s="4">
-        <v>151.644</v>
+        <v>152.334</v>
       </c>
       <c r="EA28" s="4">
-        <v>153.269</v>
+        <v>153.884</v>
       </c>
       <c r="EB28" s="4">
-        <v>153.617</v>
+        <v>154.639</v>
+      </c>
+      <c r="EC28" s="4">
+        <v>156.385</v>
       </c>
     </row>
     <row r="29">
@@ -10001,70 +10069,73 @@
         <v>108.775</v>
       </c>
       <c r="DG29" s="0">
-        <v>109.764</v>
+        <v>109.769</v>
       </c>
       <c r="DH29" s="0">
-        <v>110.418</v>
+        <v>110.403</v>
       </c>
       <c r="DI29" s="0">
-        <v>112.464</v>
+        <v>112.446</v>
       </c>
       <c r="DJ29" s="0">
-        <v>113.74</v>
+        <v>113.732</v>
       </c>
       <c r="DK29" s="0">
-        <v>116.665</v>
+        <v>116.682</v>
       </c>
       <c r="DL29" s="0">
-        <v>120.411</v>
+        <v>120.437</v>
       </c>
       <c r="DM29" s="0">
-        <v>124.696</v>
+        <v>124.716</v>
       </c>
       <c r="DN29" s="0">
-        <v>128.929</v>
+        <v>128.923</v>
       </c>
       <c r="DO29" s="0">
-        <v>134.018</v>
+        <v>133.963</v>
       </c>
       <c r="DP29" s="0">
-        <v>139.645</v>
+        <v>139.586</v>
       </c>
       <c r="DQ29" s="0">
-        <v>143.119</v>
+        <v>143.11</v>
       </c>
       <c r="DR29" s="0">
-        <v>146.132</v>
+        <v>146.247</v>
       </c>
       <c r="DS29" s="0">
-        <v>145.327</v>
+        <v>145.655</v>
       </c>
       <c r="DT29" s="0">
-        <v>144.55</v>
+        <v>144.971</v>
       </c>
       <c r="DU29" s="0">
-        <v>145.573</v>
+        <v>145.944</v>
       </c>
       <c r="DV29" s="0">
-        <v>147.674</v>
+        <v>147.862</v>
       </c>
       <c r="DW29" s="0">
-        <v>147.582</v>
+        <v>147.471</v>
       </c>
       <c r="DX29" s="0">
-        <v>149.147</v>
+        <v>148.789</v>
       </c>
       <c r="DY29" s="0">
-        <v>149.603</v>
+        <v>149.068</v>
       </c>
       <c r="DZ29" s="0">
-        <v>149.926</v>
+        <v>149.386</v>
       </c>
       <c r="EA29" s="0">
-        <v>151.974</v>
+        <v>151.68</v>
       </c>
       <c r="EB29" s="0">
-        <v>152.134</v>
+        <v>151.832</v>
+      </c>
+      <c r="EC29" s="0">
+        <v>153.036</v>
       </c>
     </row>
     <row r="30">
@@ -10399,70 +10470,73 @@
         <v>108.764</v>
       </c>
       <c r="DG30" s="0">
-        <v>109.912</v>
+        <v>109.935</v>
       </c>
       <c r="DH30" s="0">
-        <v>110.629</v>
+        <v>110.631</v>
       </c>
       <c r="DI30" s="0">
-        <v>113.098</v>
+        <v>113.087</v>
       </c>
       <c r="DJ30" s="0">
-        <v>114.603</v>
+        <v>114.59</v>
       </c>
       <c r="DK30" s="0">
-        <v>118.179</v>
+        <v>118.174</v>
       </c>
       <c r="DL30" s="0">
         <v>122.69</v>
       </c>
       <c r="DM30" s="0">
-        <v>127.807</v>
+        <v>127.81</v>
       </c>
       <c r="DN30" s="0">
-        <v>132.591</v>
+        <v>132.593</v>
       </c>
       <c r="DO30" s="0">
-        <v>138.384</v>
+        <v>138.383</v>
       </c>
       <c r="DP30" s="0">
-        <v>144.804</v>
+        <v>144.801</v>
       </c>
       <c r="DQ30" s="0">
         <v>148.531</v>
       </c>
       <c r="DR30" s="0">
-        <v>151.913</v>
+        <v>151.917</v>
       </c>
       <c r="DS30" s="0">
-        <v>150.338</v>
+        <v>150.35</v>
       </c>
       <c r="DT30" s="0">
-        <v>148.773</v>
+        <v>148.784</v>
       </c>
       <c r="DU30" s="0">
-        <v>149.858</v>
+        <v>149.857</v>
       </c>
       <c r="DV30" s="0">
-        <v>152.265</v>
+        <v>152.242</v>
       </c>
       <c r="DW30" s="0">
-        <v>151.786</v>
+        <v>151.731</v>
       </c>
       <c r="DX30" s="0">
-        <v>153.49</v>
+        <v>153.384</v>
       </c>
       <c r="DY30" s="0">
-        <v>153.676</v>
+        <v>153.527</v>
       </c>
       <c r="DZ30" s="0">
-        <v>153.676</v>
+        <v>153.625</v>
       </c>
       <c r="EA30" s="0">
-        <v>156.019</v>
+        <v>156.286</v>
       </c>
       <c r="EB30" s="0">
-        <v>155.939</v>
+        <v>156.207</v>
+      </c>
+      <c r="EC30" s="0">
+        <v>157.619</v>
       </c>
     </row>
     <row r="31">
@@ -10797,70 +10871,73 @@
         <v>108.726</v>
       </c>
       <c r="DG31" s="0">
-        <v>109.038</v>
+        <v>108.995</v>
       </c>
       <c r="DH31" s="0">
-        <v>109.399</v>
+        <v>109.342</v>
       </c>
       <c r="DI31" s="0">
-        <v>110.069</v>
+        <v>110.027</v>
       </c>
       <c r="DJ31" s="0">
-        <v>110.57</v>
+        <v>110.574</v>
       </c>
       <c r="DK31" s="0">
-        <v>111.21</v>
+        <v>111.29</v>
       </c>
       <c r="DL31" s="0">
-        <v>112.409</v>
+        <v>112.501</v>
       </c>
       <c r="DM31" s="0">
-        <v>114.073</v>
+        <v>114.108</v>
       </c>
       <c r="DN31" s="0">
-        <v>116.917</v>
+        <v>116.823</v>
       </c>
       <c r="DO31" s="0">
-        <v>120.294</v>
+        <v>119.988</v>
       </c>
       <c r="DP31" s="0">
-        <v>123.585</v>
+        <v>123.275</v>
       </c>
       <c r="DQ31" s="0">
-        <v>126.383</v>
+        <v>126.302</v>
       </c>
       <c r="DR31" s="0">
-        <v>128.106</v>
+        <v>128.5</v>
       </c>
       <c r="DS31" s="0">
-        <v>128.824</v>
+        <v>129.945</v>
       </c>
       <c r="DT31" s="0">
-        <v>129.654</v>
+        <v>131.115</v>
       </c>
       <c r="DU31" s="0">
-        <v>130.261</v>
+        <v>131.667</v>
       </c>
       <c r="DV31" s="0">
-        <v>131.364</v>
+        <v>132.316</v>
       </c>
       <c r="DW31" s="0">
-        <v>132.369</v>
+        <v>132.448</v>
       </c>
       <c r="DX31" s="0">
-        <v>133.496</v>
+        <v>132.907</v>
       </c>
       <c r="DY31" s="0">
-        <v>134.732</v>
+        <v>133.685</v>
       </c>
       <c r="DZ31" s="0">
-        <v>136.026</v>
+        <v>134.74</v>
       </c>
       <c r="EA31" s="0">
-        <v>137.117</v>
+        <v>135.821</v>
       </c>
       <c r="EB31" s="0">
-        <v>138.035</v>
+        <v>136.729</v>
+      </c>
+      <c r="EC31" s="0">
+        <v>137.253</v>
       </c>
     </row>
     <row r="32">
@@ -11195,70 +11272,73 @@
         <v>110.842</v>
       </c>
       <c r="DG32" s="0">
-        <v>111.199</v>
+        <v>111.634</v>
       </c>
       <c r="DH32" s="0">
-        <v>110.903</v>
+        <v>111.173</v>
       </c>
       <c r="DI32" s="0">
-        <v>113.736</v>
+        <v>114.156</v>
       </c>
       <c r="DJ32" s="0">
-        <v>116.133</v>
+        <v>116.894</v>
       </c>
       <c r="DK32" s="0">
-        <v>119.837</v>
+        <v>120.752</v>
       </c>
       <c r="DL32" s="0">
-        <v>124.472</v>
+        <v>125.913</v>
       </c>
       <c r="DM32" s="0">
-        <v>128.952</v>
+        <v>130.239</v>
       </c>
       <c r="DN32" s="0">
-        <v>132.372</v>
+        <v>133.414</v>
       </c>
       <c r="DO32" s="0">
-        <v>138.456</v>
+        <v>139.135</v>
       </c>
       <c r="DP32" s="0">
-        <v>142.633</v>
+        <v>143.124</v>
       </c>
       <c r="DQ32" s="0">
-        <v>145.313</v>
+        <v>144.862</v>
       </c>
       <c r="DR32" s="0">
-        <v>146.314</v>
+        <v>145.493</v>
       </c>
       <c r="DS32" s="0">
-        <v>145.022</v>
+        <v>143.567</v>
       </c>
       <c r="DT32" s="0">
-        <v>145.021</v>
+        <v>143.64</v>
       </c>
       <c r="DU32" s="0">
-        <v>147.609</v>
+        <v>146.911</v>
       </c>
       <c r="DV32" s="0">
-        <v>148.89</v>
+        <v>148.232</v>
       </c>
       <c r="DW32" s="0">
-        <v>148.613</v>
+        <v>149.009</v>
       </c>
       <c r="DX32" s="0">
-        <v>149.782</v>
+        <v>150.379</v>
       </c>
       <c r="DY32" s="0">
-        <v>151.864</v>
+        <v>153.18</v>
       </c>
       <c r="DZ32" s="0">
-        <v>152.983</v>
+        <v>154.784</v>
       </c>
       <c r="EA32" s="0">
-        <v>154.231</v>
+        <v>155.669</v>
       </c>
       <c r="EB32" s="0">
-        <v>154.742</v>
+        <v>156.954</v>
+      </c>
+      <c r="EC32" s="0">
+        <v>159.167</v>
       </c>
     </row>
     <row r="33">
@@ -11593,70 +11673,73 @@
         <v>101.847</v>
       </c>
       <c r="DG33" s="4">
-        <v>102.493</v>
+        <v>102.736</v>
       </c>
       <c r="DH33" s="4">
-        <v>104.78</v>
+        <v>104.608</v>
       </c>
       <c r="DI33" s="4">
-        <v>109.831</v>
+        <v>109.652</v>
       </c>
       <c r="DJ33" s="4">
-        <v>113.818</v>
+        <v>113.839</v>
       </c>
       <c r="DK33" s="4">
-        <v>113.097</v>
+        <v>113.269</v>
       </c>
       <c r="DL33" s="4">
-        <v>115.525</v>
+        <v>115.472</v>
       </c>
       <c r="DM33" s="4">
-        <v>119.324</v>
+        <v>119.16</v>
       </c>
       <c r="DN33" s="4">
-        <v>121.641</v>
+        <v>121.667</v>
       </c>
       <c r="DO33" s="4">
-        <v>125.263</v>
+        <v>125.424</v>
       </c>
       <c r="DP33" s="4">
-        <v>126.661</v>
+        <v>126.73</v>
       </c>
       <c r="DQ33" s="4">
-        <v>124.248</v>
+        <v>124.03</v>
       </c>
       <c r="DR33" s="4">
-        <v>123.653</v>
+        <v>123.602</v>
       </c>
       <c r="DS33" s="4">
-        <v>121.375</v>
+        <v>121.508</v>
       </c>
       <c r="DT33" s="4">
-        <v>117.819</v>
+        <v>117.989</v>
       </c>
       <c r="DU33" s="4">
-        <v>115.855</v>
+        <v>115.607</v>
       </c>
       <c r="DV33" s="4">
-        <v>113.675</v>
+        <v>113.592</v>
       </c>
       <c r="DW33" s="4">
-        <v>114.471</v>
+        <v>114.553</v>
       </c>
       <c r="DX33" s="4">
-        <v>111.986</v>
+        <v>112.28</v>
       </c>
       <c r="DY33" s="4">
-        <v>112.449</v>
+        <v>112.266</v>
       </c>
       <c r="DZ33" s="4">
-        <v>111.445</v>
+        <v>111.014</v>
       </c>
       <c r="EA33" s="4">
-        <v>108.885</v>
+        <v>108.47</v>
       </c>
       <c r="EB33" s="4">
-        <v>112.227</v>
+        <v>111.797</v>
+      </c>
+      <c r="EC33" s="4">
+        <v>112.239</v>
       </c>
     </row>
     <row r="34">
@@ -12056,6 +12139,9 @@
       <c r="EB34" s="0" t="s">
         <v>5</v>
       </c>
+      <c r="EC34" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="s">
@@ -12389,70 +12475,73 @@
         <v>108.424</v>
       </c>
       <c r="DG35" s="0">
-        <v>109.076</v>
+        <v>109.208</v>
       </c>
       <c r="DH35" s="0">
-        <v>108.935</v>
+        <v>109.043</v>
       </c>
       <c r="DI35" s="0">
-        <v>110.266</v>
+        <v>110.418</v>
       </c>
       <c r="DJ35" s="0">
-        <v>111.249</v>
+        <v>111.539</v>
       </c>
       <c r="DK35" s="0">
-        <v>113.312</v>
+        <v>113.625</v>
       </c>
       <c r="DL35" s="0">
-        <v>116.467</v>
+        <v>116.968</v>
       </c>
       <c r="DM35" s="0">
-        <v>120.033</v>
+        <v>120.471</v>
       </c>
       <c r="DN35" s="0">
-        <v>124.68</v>
+        <v>125.084</v>
       </c>
       <c r="DO35" s="0">
-        <v>129.911</v>
+        <v>130.19</v>
       </c>
       <c r="DP35" s="0">
-        <v>134.879</v>
+        <v>135.147</v>
       </c>
       <c r="DQ35" s="0">
-        <v>138.781</v>
+        <v>138.756</v>
       </c>
       <c r="DR35" s="0">
-        <v>141.036</v>
+        <v>140.966</v>
       </c>
       <c r="DS35" s="0">
-        <v>141.375</v>
+        <v>141.035</v>
       </c>
       <c r="DT35" s="0">
-        <v>141.017</v>
+        <v>140.74</v>
       </c>
       <c r="DU35" s="0">
-        <v>141.377</v>
+        <v>141.223</v>
       </c>
       <c r="DV35" s="0">
-        <v>142.811</v>
+        <v>142.641</v>
       </c>
       <c r="DW35" s="0">
-        <v>142.385</v>
+        <v>142.349</v>
       </c>
       <c r="DX35" s="0">
-        <v>143.168</v>
+        <v>143.341</v>
       </c>
       <c r="DY35" s="0">
-        <v>144.156</v>
+        <v>144.058</v>
       </c>
       <c r="DZ35" s="0">
-        <v>144.456</v>
+        <v>144.637</v>
       </c>
       <c r="EA35" s="0">
-        <v>145.72</v>
+        <v>145.632</v>
       </c>
       <c r="EB35" s="0">
-        <v>145.791</v>
+        <v>145.871</v>
+      </c>
+      <c r="EC35" s="0">
+        <v>147.369</v>
       </c>
     </row>
     <row r="36">
@@ -12787,70 +12876,73 @@
         <v>107.501</v>
       </c>
       <c r="DG36" s="0">
-        <v>108.202</v>
+        <v>108.349</v>
       </c>
       <c r="DH36" s="0">
-        <v>107.913</v>
+        <v>108.035</v>
       </c>
       <c r="DI36" s="0">
-        <v>109.131</v>
+        <v>109.301</v>
       </c>
       <c r="DJ36" s="0">
-        <v>109.771</v>
+        <v>110.096</v>
       </c>
       <c r="DK36" s="0">
-        <v>111.597</v>
+        <v>111.944</v>
       </c>
       <c r="DL36" s="0">
-        <v>114.715</v>
+        <v>115.28</v>
       </c>
       <c r="DM36" s="0">
-        <v>118.032</v>
+        <v>118.523</v>
       </c>
       <c r="DN36" s="0">
-        <v>123.164</v>
+        <v>123.625</v>
       </c>
       <c r="DO36" s="0">
-        <v>128.425</v>
+        <v>128.743</v>
       </c>
       <c r="DP36" s="0">
-        <v>133.946</v>
+        <v>134.25</v>
       </c>
       <c r="DQ36" s="0">
-        <v>137.876</v>
+        <v>137.845</v>
       </c>
       <c r="DR36" s="0">
-        <v>140.451</v>
+        <v>140.368</v>
       </c>
       <c r="DS36" s="0">
-        <v>140.979</v>
+        <v>140.582</v>
       </c>
       <c r="DT36" s="0">
-        <v>140.34</v>
+        <v>140.019</v>
       </c>
       <c r="DU36" s="0">
-        <v>140.252</v>
+        <v>140.079</v>
       </c>
       <c r="DV36" s="0">
-        <v>141.802</v>
+        <v>141.608</v>
       </c>
       <c r="DW36" s="0">
-        <v>141.556</v>
+        <v>141.489</v>
       </c>
       <c r="DX36" s="0">
-        <v>142.188</v>
+        <v>142.36</v>
       </c>
       <c r="DY36" s="0">
-        <v>142.956</v>
+        <v>142.837</v>
       </c>
       <c r="DZ36" s="0">
-        <v>143.256</v>
+        <v>143.446</v>
       </c>
       <c r="EA36" s="0">
-        <v>144.684</v>
+        <v>144.567</v>
       </c>
       <c r="EB36" s="0">
-        <v>144.619</v>
+        <v>144.689</v>
+      </c>
+      <c r="EC36" s="0">
+        <v>145.978</v>
       </c>
     </row>
     <row r="37">
@@ -13185,70 +13277,73 @@
         <v>106.458</v>
       </c>
       <c r="DG37" s="0">
-        <v>107.138</v>
+        <v>107.134</v>
       </c>
       <c r="DH37" s="0">
-        <v>106.672</v>
+        <v>106.742</v>
       </c>
       <c r="DI37" s="0">
-        <v>106.479</v>
+        <v>106.546</v>
       </c>
       <c r="DJ37" s="0">
-        <v>106.067</v>
+        <v>106.199</v>
       </c>
       <c r="DK37" s="0">
-        <v>106.069</v>
+        <v>106.121</v>
       </c>
       <c r="DL37" s="0">
-        <v>107.701</v>
+        <v>107.827</v>
       </c>
       <c r="DM37" s="0">
-        <v>109.986</v>
+        <v>110.083</v>
       </c>
       <c r="DN37" s="0">
-        <v>116.242</v>
+        <v>116.482</v>
       </c>
       <c r="DO37" s="0">
-        <v>121.105</v>
+        <v>121.356</v>
       </c>
       <c r="DP37" s="0">
-        <v>126.461</v>
+        <v>126.828</v>
       </c>
       <c r="DQ37" s="0">
-        <v>131.726</v>
+        <v>131.996</v>
       </c>
       <c r="DR37" s="0">
-        <v>134.427</v>
+        <v>134.737</v>
       </c>
       <c r="DS37" s="0">
-        <v>136.577</v>
+        <v>136.476</v>
       </c>
       <c r="DT37" s="0">
-        <v>136.292</v>
+        <v>136.194</v>
       </c>
       <c r="DU37" s="0">
-        <v>134.925</v>
+        <v>134.779</v>
       </c>
       <c r="DV37" s="0">
-        <v>136.199</v>
+        <v>136.095</v>
       </c>
       <c r="DW37" s="0">
-        <v>135.689</v>
+        <v>135.417</v>
       </c>
       <c r="DX37" s="0">
-        <v>135.798</v>
+        <v>136.039</v>
       </c>
       <c r="DY37" s="0">
-        <v>136.355</v>
+        <v>135.699</v>
       </c>
       <c r="DZ37" s="0">
-        <v>136.122</v>
+        <v>135.806</v>
       </c>
       <c r="EA37" s="0">
-        <v>137.002</v>
+        <v>136.171</v>
       </c>
       <c r="EB37" s="0">
-        <v>136.741</v>
+        <v>135.799</v>
+      </c>
+      <c r="EC37" s="0">
+        <v>137.03</v>
       </c>
     </row>
     <row r="38">
@@ -13583,70 +13678,73 @@
         <v>108.503</v>
       </c>
       <c r="DG38" s="0">
-        <v>109.265</v>
+        <v>109.558</v>
       </c>
       <c r="DH38" s="0">
-        <v>109.179</v>
+        <v>109.351</v>
       </c>
       <c r="DI38" s="0">
-        <v>111.635</v>
+        <v>111.901</v>
       </c>
       <c r="DJ38" s="0">
-        <v>113.136</v>
+        <v>113.637</v>
       </c>
       <c r="DK38" s="0">
-        <v>116.38</v>
+        <v>116.99</v>
       </c>
       <c r="DL38" s="0">
-        <v>120.653</v>
+        <v>121.598</v>
       </c>
       <c r="DM38" s="0">
-        <v>124.778</v>
+        <v>125.623</v>
       </c>
       <c r="DN38" s="0">
-        <v>129.106</v>
+        <v>129.79</v>
       </c>
       <c r="DO38" s="0">
-        <v>134.694</v>
+        <v>135.122</v>
       </c>
       <c r="DP38" s="0">
-        <v>140.368</v>
+        <v>140.68</v>
       </c>
       <c r="DQ38" s="0">
-        <v>143.22</v>
+        <v>142.991</v>
       </c>
       <c r="DR38" s="0">
-        <v>145.68</v>
+        <v>145.302</v>
       </c>
       <c r="DS38" s="0">
-        <v>144.66</v>
+        <v>144.01</v>
       </c>
       <c r="DT38" s="0">
-        <v>143.666</v>
+        <v>143.131</v>
       </c>
       <c r="DU38" s="0">
-        <v>144.825</v>
+        <v>144.677</v>
       </c>
       <c r="DV38" s="0">
-        <v>146.631</v>
+        <v>146.409</v>
       </c>
       <c r="DW38" s="0">
-        <v>146.64</v>
+        <v>146.863</v>
       </c>
       <c r="DX38" s="0">
-        <v>147.77</v>
+        <v>147.984</v>
       </c>
       <c r="DY38" s="0">
-        <v>148.738</v>
+        <v>149.278</v>
       </c>
       <c r="DZ38" s="0">
-        <v>149.546</v>
+        <v>150.383</v>
       </c>
       <c r="EA38" s="0">
-        <v>151.493</v>
+        <v>152.237</v>
       </c>
       <c r="EB38" s="0">
-        <v>151.614</v>
+        <v>152.834</v>
+      </c>
+      <c r="EC38" s="0">
+        <v>154.176</v>
       </c>
     </row>
     <row r="39">
@@ -13981,70 +14079,73 @@
         <v>94.026</v>
       </c>
       <c r="DG39" s="0">
-        <v>93.478</v>
+        <v>93.487</v>
       </c>
       <c r="DH39" s="0">
-        <v>93.234</v>
+        <v>93.241</v>
       </c>
       <c r="DI39" s="0">
-        <v>92.948</v>
+        <v>92.951</v>
       </c>
       <c r="DJ39" s="0">
-        <v>92.824</v>
+        <v>92.816</v>
       </c>
       <c r="DK39" s="0">
-        <v>91.695</v>
+        <v>91.664</v>
       </c>
       <c r="DL39" s="0">
-        <v>91.641</v>
+        <v>91.593</v>
       </c>
       <c r="DM39" s="0">
-        <v>91.527</v>
+        <v>91.459</v>
       </c>
       <c r="DN39" s="0">
-        <v>91.361</v>
+        <v>91.266</v>
       </c>
       <c r="DO39" s="0">
-        <v>91.303</v>
+        <v>91.168</v>
       </c>
       <c r="DP39" s="0">
-        <v>91.448</v>
+        <v>91.299</v>
       </c>
       <c r="DQ39" s="0">
-        <v>91.657</v>
+        <v>91.509</v>
       </c>
       <c r="DR39" s="0">
-        <v>91.002</v>
+        <v>90.868</v>
       </c>
       <c r="DS39" s="0">
-        <v>92.26</v>
+        <v>92.151</v>
       </c>
       <c r="DT39" s="0">
-        <v>91.999</v>
+        <v>91.894</v>
       </c>
       <c r="DU39" s="0">
-        <v>91.886</v>
+        <v>91.7</v>
       </c>
       <c r="DV39" s="0">
-        <v>91.832</v>
+        <v>91.528</v>
       </c>
       <c r="DW39" s="0">
-        <v>91.985</v>
+        <v>91.512</v>
       </c>
       <c r="DX39" s="0">
-        <v>93.055</v>
+        <v>92.45</v>
       </c>
       <c r="DY39" s="0">
-        <v>94.195</v>
+        <v>93.499</v>
       </c>
       <c r="DZ39" s="0">
-        <v>94.587</v>
+        <v>93.842</v>
       </c>
       <c r="EA39" s="0">
-        <v>93.731</v>
+        <v>92.836</v>
       </c>
       <c r="EB39" s="0">
-        <v>92.23</v>
+        <v>91.548</v>
+      </c>
+      <c r="EC39" s="0">
+        <v>93.189</v>
       </c>
     </row>
     <row r="40">
@@ -14099,10 +14200,10 @@
     </row>
   </sheetData>
   <mergeCells>
-    <mergeCell ref="A1:EB1"/>
-    <mergeCell ref="A2:EB2"/>
-    <mergeCell ref="A3:EB3"/>
-    <mergeCell ref="A4:EB4"/>
+    <mergeCell ref="A1:EC1"/>
+    <mergeCell ref="A2:EC2"/>
+    <mergeCell ref="A3:EC3"/>
+    <mergeCell ref="A4:EC4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="C6:F6"/>
@@ -14137,17 +14238,17 @@
     <mergeCell ref="DO6:DR6"/>
     <mergeCell ref="DS6:DV6"/>
     <mergeCell ref="DW6:DZ6"/>
-    <mergeCell ref="EA6:EB6"/>
-    <mergeCell ref="A40:EC40"/>
-    <mergeCell ref="A41:EC41"/>
-    <mergeCell ref="A42:EC42"/>
-    <mergeCell ref="A43:EC43"/>
-    <mergeCell ref="A44:EC44"/>
-    <mergeCell ref="A45:EC45"/>
-    <mergeCell ref="A46:EC46"/>
-    <mergeCell ref="A47:EC47"/>
-    <mergeCell ref="A48:EC48"/>
-    <mergeCell ref="A49:EC49"/>
+    <mergeCell ref="EA6:EC6"/>
+    <mergeCell ref="A40:ED40"/>
+    <mergeCell ref="A41:ED41"/>
+    <mergeCell ref="A42:ED42"/>
+    <mergeCell ref="A43:ED43"/>
+    <mergeCell ref="A44:ED44"/>
+    <mergeCell ref="A45:ED45"/>
+    <mergeCell ref="A46:ED46"/>
+    <mergeCell ref="A47:ED47"/>
+    <mergeCell ref="A48:ED48"/>
+    <mergeCell ref="A49:ED49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>